<commit_message>
remplazo de archivo de carga masiva
</commit_message>
<xml_diff>
--- a/Frontend/public/TablaCargaMasiva.xlsx
+++ b/Frontend/public/TablaCargaMasiva.xlsx
@@ -630,7 +630,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>equipos</t>
+          <t>Equipamiento</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>equipos</t>
+          <t>Equipamiento</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1085,6 +1085,11 @@
       <c r="R10" s="4" t="n"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Categoría inválida" error="Seleccioná una categoría de la lista: Insumos, Procesos, Equipamiento, Mobiliario." promptTitle="Categoría nivel 0" prompt="Seleccioná la categoría raíz del producto." type="list">
+      <formula1>"Insumos,Procesos,Equipamiento,Mobiliario"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1142,7 +1147,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   categoria_nivel_0      Categoria raiz — valores validos: insumos, procesos, equipos, mobiliario</t>
+          <t xml:space="preserve">   categoria_nivel_0      Categoria raiz — debe coincidir con una categoria existente en la base de datos (ej: Insumos, Procesos, Equipamiento, Mobiliario)</t>
         </is>
       </c>
     </row>
@@ -1494,21 +1499,21 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ERROR: Fila N: error al procesar producto "X" — Categoria nivel 0 invalida</t>
+          <t xml:space="preserve">   ERROR: Fila N: error al procesar producto "X" — Categoria nivel 0 no encontrada</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Causa:    El valor de categoria_nivel_0 no es uno de los permitidos.</t>
+          <t xml:space="preserve">   Causa:    El valor de categoria_nivel_0 no coincide con ninguna categoria raiz en la base de datos.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Solucion: Usar solo: insumos, procesos, equipos, mobiliario (exactamente, sin tildes).</t>
+          <t xml:space="preserve">   Solucion: Verificar el nombre exacto de la categoria raiz en el sistema (ej: Insumos, Procesos, Equipamiento, Mobiliario).</t>
         </is>
       </c>
     </row>

</xml_diff>